<commit_message>
feat: add lined channel Excel exports
</commit_message>
<xml_diff>
--- a/templates/excel/form_2_2_V1.xlsx
+++ b/templates/excel/form_2_2_V1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\gitProject\YindaSurveySystem\templates\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30C727F5-FBFB-429A-9968-CB647CA8BA45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A4A1BEE-3790-400C-A95A-7CDD78572A17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15264" yWindow="0" windowWidth="15552" windowHeight="16656" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="附表2.2" sheetId="1" r:id="rId1"/>
@@ -85,137 +85,137 @@
     <t>项目</t>
   </si>
   <si>
+    <t>项目类别</t>
+  </si>
+  <si>
+    <t>情况描述</t>
+  </si>
+  <si>
+    <t>水力条件</t>
+  </si>
+  <si>
+    <t>进、出口流态</t>
+  </si>
+  <si>
+    <t>a 闸室进、出口流态平稳。b 闸室进、出口流态基本平稳。c 闸室进、出口流态不稳，出现连续非贯穿性漩涡。d 闸室进、出口流态紊乱，出现连续贯穿性漩涡。</t>
+  </si>
+  <si>
+    <t>上、下游水位</t>
+  </si>
+  <si>
+    <t>a 闸室水位满足设计要求。b 闸室水位降小于设计水深的5%。c 闸室水位降为设计水深的5%～10%。d 闸室水位降大于设计水深的10%。</t>
+  </si>
+  <si>
+    <t>过闸流量</t>
+  </si>
+  <si>
+    <t>a 过闸流量符合设计要求。b 过闸流量为设计值的95%以上。c 过闸流量为设计值的90%～95%。d 过闸流量为设计值的90%以下。</t>
+  </si>
+  <si>
+    <t>闸后消能与冲刷</t>
+  </si>
+  <si>
+    <t>a 闸后泄槽流态平稳，消能充分。b 闸后泄槽流态基本平稳，无冲刷破坏。c 闸后泄槽流态紊乱，消能不充分，防冲设施冲刷破坏。d 闸后泄槽流态紊乱，防冲设施冲刷破坏严重，危及工程安全。</t>
+  </si>
+  <si>
+    <t>结构变形</t>
+  </si>
+  <si>
+    <t>进口翼墙</t>
+  </si>
+  <si>
+    <t>a 结构变形符合设计要求。b 闸室边墙及闸墩的变位，不影响闸门正常升降。c 闸室边墙及闸墩的变位影响闸门正常升降。d 闸室边墙及闸墩的变位造成闸门不能正常升降，危及工程安全。</t>
+  </si>
+  <si>
+    <t>闸室</t>
+  </si>
+  <si>
+    <t>a 泄槽表面平整度符合设计要求。b 泄槽表面平整度小于20mm。c 泄槽表面平整度为20mm～40mm。d 泄槽表面平整度大于40mm。</t>
+  </si>
+  <si>
+    <t>消能设施</t>
+  </si>
+  <si>
+    <t>a 其它部位结构变形符合设计要求。b 其它部位结构变形不影响工程正常运行。c 其它部位结构变形影响工程正常运行。d 其它部位结构变形危及工程安全。</t>
+  </si>
+  <si>
+    <t>结构破损</t>
+  </si>
+  <si>
+    <t>a 闸室结构完好。b 闸室局部有剥蚀现象；裂缝短小、不跨层，裂缝宽度小于0.2mm。c 闸室有贯穿性裂缝，裂缝宽度为0.2mm～0.3mm；结构破损，钢筋锈蚀。d 闸室有贯穿性裂缝，裂缝宽度大于0.3mm；表面剥蚀，钢筋锈蚀程度危及工程安全。</t>
+  </si>
+  <si>
+    <t>a 消能设施完好。b 消能设施冲蚀、裂缝刚发生。c 消能设施冲蚀、裂缝扩展。d 消能设施破损危及工程安全。</t>
+  </si>
+  <si>
+    <t>其它部位</t>
+  </si>
+  <si>
+    <t>a 其它部位结构完好。b 其它部位有剥蚀和裂缝现象。c 其它部位有贯穿性裂缝、表层有剥蚀、脱落现象。d 其它部位结构不完整。</t>
+  </si>
+  <si>
+    <t>混凝土碳化深度</t>
+  </si>
+  <si>
+    <t>a 混凝土碳化深度小于钢筋保护层厚度。b 混凝土碳化深度小于钢筋保护层厚度。c 混凝土碳化深度达到钢筋保护层厚度。d 混凝土碳化深度大于钢筋保护层厚度。</t>
+  </si>
+  <si>
+    <t>a 混凝土强度符合设计要求。b 混凝土强度为设计值的90%以上。c 混凝土强度为设计值的80%～90%。d 混凝土强度为设计值80%以下。</t>
+  </si>
+  <si>
+    <t>地基基础</t>
+  </si>
+  <si>
+    <t>地基</t>
+  </si>
+  <si>
+    <t>a 闸底板无变形。b 闸底板变形、裂缝刚发生。c 闸基础倾斜，底板裂缝扩展，闸后有渗水或清水逸出。d 闸基础倾斜，底板裂缝，闸后有浑水逸出。</t>
+  </si>
+  <si>
+    <t>基础</t>
+  </si>
+  <si>
+    <t>a 基础无变形。b 基础胀沉小于50mm。c 基础胀沉为50mm～80mm。d 基础胀沉大于80mm。</t>
+  </si>
+  <si>
+    <t>调查意见与建议</t>
+  </si>
+  <si>
+    <t>工程状况类别</t>
+  </si>
+  <si>
+    <t>调查人签字</t>
+  </si>
+  <si>
+    <t>水管所负责人</t>
+  </si>
+  <si>
+    <t>工程科科长</t>
+  </si>
+  <si>
+    <t>基层处负责人</t>
+  </si>
+  <si>
+    <t>调查时间</t>
+  </si>
+  <si>
+    <t>注：1. 进水闸（节制闸、分水闸）其它部位包括进出口衔接段及消能设施、沉沙池等，无泄槽流态、泄槽表面平整度要求。</t>
+  </si>
+  <si>
+    <t>2. 泄洪闸（退水闸）其它部位指闸室进出口渐变段、泄槽及消能设施等，无闸室水位降要求。</t>
+  </si>
+  <si>
     <t>序号</t>
   </si>
   <si>
-    <t>检查部位与内容</t>
-  </si>
-  <si>
-    <t>项目类别</t>
-  </si>
-  <si>
-    <t>情况描述</t>
-  </si>
-  <si>
-    <t>水力条件</t>
-  </si>
-  <si>
-    <t>进、出口流态</t>
-  </si>
-  <si>
-    <t>a 闸室进、出口流态平稳。b 闸室进、出口流态基本平稳。c 闸室进、出口流态不稳，出现连续非贯穿性漩涡。d 闸室进、出口流态紊乱，出现连续贯穿性漩涡。</t>
-  </si>
-  <si>
-    <t>上、下游水位</t>
-  </si>
-  <si>
-    <t>a 闸室水位满足设计要求。b 闸室水位降小于设计水深的5%。c 闸室水位降为设计水深的5%～10%。d 闸室水位降大于设计水深的10%。</t>
-  </si>
-  <si>
-    <t>过闸流量</t>
-  </si>
-  <si>
-    <t>a 过闸流量符合设计要求。b 过闸流量为设计值的95%以上。c 过闸流量为设计值的90%～95%。d 过闸流量为设计值的90%以下。</t>
-  </si>
-  <si>
-    <t>闸后消能与冲刷</t>
-  </si>
-  <si>
-    <t>a 闸后泄槽流态平稳，消能充分。b 闸后泄槽流态基本平稳，无冲刷破坏。c 闸后泄槽流态紊乱，消能不充分，防冲设施冲刷破坏。d 闸后泄槽流态紊乱，防冲设施冲刷破坏严重，危及工程安全。</t>
-  </si>
-  <si>
-    <t>结构变形</t>
-  </si>
-  <si>
-    <t>进口翼墙</t>
-  </si>
-  <si>
-    <t>a 结构变形符合设计要求。b 闸室边墙及闸墩的变位，不影响闸门正常升降。c 闸室边墙及闸墩的变位影响闸门正常升降。d 闸室边墙及闸墩的变位造成闸门不能正常升降，危及工程安全。</t>
-  </si>
-  <si>
-    <t>闸室</t>
-  </si>
-  <si>
-    <t>a 泄槽表面平整度符合设计要求。b 泄槽表面平整度小于20mm。c 泄槽表面平整度为20mm～40mm。d 泄槽表面平整度大于40mm。</t>
-  </si>
-  <si>
-    <t>消能设施</t>
-  </si>
-  <si>
-    <t>a 其它部位结构变形符合设计要求。b 其它部位结构变形不影响工程正常运行。c 其它部位结构变形影响工程正常运行。d 其它部位结构变形危及工程安全。</t>
-  </si>
-  <si>
-    <t>结构破损</t>
-  </si>
-  <si>
-    <t>a 闸室结构完好。b 闸室局部有剥蚀现象；裂缝短小、不跨层，裂缝宽度小于0.2mm。c 闸室有贯穿性裂缝，裂缝宽度为0.2mm～0.3mm；结构破损，钢筋锈蚀。d 闸室有贯穿性裂缝，裂缝宽度大于0.3mm；表面剥蚀，钢筋锈蚀程度危及工程安全。</t>
-  </si>
-  <si>
-    <t>a 消能设施完好。b 消能设施冲蚀、裂缝刚发生。c 消能设施冲蚀、裂缝扩展。d 消能设施破损危及工程安全。</t>
-  </si>
-  <si>
-    <t>其它部位</t>
-  </si>
-  <si>
-    <t>a 其它部位结构完好。b 其它部位有剥蚀和裂缝现象。c 其它部位有贯穿性裂缝、表层有剥蚀、脱落现象。d 其它部位结构不完整。</t>
-  </si>
-  <si>
-    <t>混凝土碳化深度</t>
-  </si>
-  <si>
-    <t>a 混凝土碳化深度小于钢筋保护层厚度。b 混凝土碳化深度小于钢筋保护层厚度。c 混凝土碳化深度达到钢筋保护层厚度。d 混凝土碳化深度大于钢筋保护层厚度。</t>
-  </si>
-  <si>
-    <t>a 混凝土强度符合设计要求。b 混凝土强度为设计值的90%以上。c 混凝土强度为设计值的80%～90%。d 混凝土强度为设计值80%以下。</t>
-  </si>
-  <si>
-    <t>地基基础</t>
-  </si>
-  <si>
-    <t>地基</t>
-  </si>
-  <si>
-    <t>a 闸底板无变形。b 闸底板变形、裂缝刚发生。c 闸基础倾斜，底板裂缝扩展，闸后有渗水或清水逸出。d 闸基础倾斜，底板裂缝，闸后有浑水逸出。</t>
-  </si>
-  <si>
-    <t>基础</t>
-  </si>
-  <si>
-    <t>a 基础无变形。b 基础胀沉小于50mm。c 基础胀沉为50mm～80mm。d 基础胀沉大于80mm。</t>
-  </si>
-  <si>
-    <t>调查意见与建议</t>
-  </si>
-  <si>
-    <t>工程状况类别</t>
-  </si>
-  <si>
-    <t>调查人签字</t>
-  </si>
-  <si>
-    <t>水管所负责人</t>
-  </si>
-  <si>
-    <t>工程科科长</t>
-  </si>
-  <si>
-    <t>基层处负责人</t>
-  </si>
-  <si>
-    <t>调查时间</t>
-  </si>
-  <si>
-    <t>注：1. 进水闸（节制闸、分水闸）其它部位包括进出口衔接段及消能设施、沉沙池等，无泄槽流态、泄槽表面平整度要求。</t>
-  </si>
-  <si>
-    <t>2. 泄洪闸（退水闸）其它部位指闸室进出口渐变段、泄槽及消能设施等，无闸室水位降要求。</t>
+    <t>检查部位及内容</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -276,6 +276,13 @@
       <family val="3"/>
       <charset val="134"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -285,7 +292,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -308,12 +315,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -350,6 +372,18 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -604,17 +638,21 @@
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
     </row>
-    <row r="3" spans="1:10" ht="19.2" customHeight="1">
-      <c r="B3" s="2" t="s">
+    <row r="3" spans="1:10">
+      <c r="A3" s="15"/>
+      <c r="B3" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="C3" s="15"/>
+      <c r="D3" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="E3" s="15"/>
+      <c r="F3" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="G3" s="15"/>
+      <c r="H3" s="16" t="s">
         <v>5</v>
       </c>
       <c r="I3" s="2" t="s">
@@ -700,18 +738,18 @@
       <c r="A8" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" s="14"/>
+      <c r="E8" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="F8" s="9" t="s">
         <v>22</v>
-      </c>
-      <c r="D8" s="9"/>
-      <c r="E8" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>24</v>
       </c>
       <c r="G8" s="9"/>
       <c r="H8" s="9"/>
@@ -720,18 +758,18 @@
     </row>
     <row r="9" spans="1:10" ht="27.15" customHeight="1">
       <c r="A9" s="8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B9" s="4">
         <v>1</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D9" s="8"/>
       <c r="E9" s="4"/>
       <c r="F9" s="10" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G9" s="10"/>
       <c r="H9" s="10"/>
@@ -744,12 +782,12 @@
         <v>2</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D10" s="8"/>
       <c r="E10" s="4"/>
       <c r="F10" s="10" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G10" s="10"/>
       <c r="H10" s="10"/>
@@ -762,12 +800,12 @@
         <v>3</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D11" s="8"/>
       <c r="E11" s="4"/>
       <c r="F11" s="10" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G11" s="10"/>
       <c r="H11" s="10"/>
@@ -780,12 +818,12 @@
         <v>4</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D12" s="8"/>
       <c r="E12" s="4"/>
       <c r="F12" s="10" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G12" s="10"/>
       <c r="H12" s="10"/>
@@ -794,18 +832,18 @@
     </row>
     <row r="13" spans="1:10" ht="27.15" customHeight="1">
       <c r="A13" s="8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B13" s="4">
         <v>1</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D13" s="8"/>
       <c r="E13" s="4"/>
       <c r="F13" s="10" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G13" s="10"/>
       <c r="H13" s="10"/>
@@ -818,12 +856,12 @@
         <v>2</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D14" s="8"/>
       <c r="E14" s="4"/>
       <c r="F14" s="10" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G14" s="10"/>
       <c r="H14" s="10"/>
@@ -836,12 +874,12 @@
         <v>3</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D15" s="8"/>
       <c r="E15" s="4"/>
       <c r="F15" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G15" s="10"/>
       <c r="H15" s="10"/>
@@ -850,18 +888,18 @@
     </row>
     <row r="16" spans="1:10" ht="27.15" customHeight="1">
       <c r="A16" s="8" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B16" s="4">
         <v>1</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D16" s="8"/>
       <c r="E16" s="4"/>
       <c r="F16" s="10" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G16" s="10"/>
       <c r="H16" s="10"/>
@@ -874,12 +912,12 @@
         <v>2</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D17" s="8"/>
       <c r="E17" s="4"/>
       <c r="F17" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="G17" s="10"/>
       <c r="H17" s="10"/>
@@ -892,12 +930,12 @@
         <v>3</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D18" s="8"/>
       <c r="E18" s="4"/>
       <c r="F18" s="10" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G18" s="10"/>
       <c r="H18" s="10"/>
@@ -910,12 +948,12 @@
         <v>4</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D19" s="8"/>
       <c r="E19" s="4"/>
       <c r="F19" s="10" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G19" s="10"/>
       <c r="H19" s="10"/>
@@ -933,7 +971,7 @@
       <c r="D20" s="8"/>
       <c r="E20" s="4"/>
       <c r="F20" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G20" s="10"/>
       <c r="H20" s="10"/>
@@ -942,18 +980,18 @@
     </row>
     <row r="21" spans="1:10" ht="27.15" customHeight="1">
       <c r="A21" s="8" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B21" s="4">
         <v>1</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D21" s="8"/>
       <c r="E21" s="4"/>
       <c r="F21" s="10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G21" s="10"/>
       <c r="H21" s="10"/>
@@ -966,12 +1004,12 @@
         <v>2</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D22" s="8"/>
       <c r="E22" s="4"/>
       <c r="F22" s="10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G22" s="10"/>
       <c r="H22" s="10"/>
@@ -980,7 +1018,7 @@
     </row>
     <row r="23" spans="1:10" ht="18.45" customHeight="1">
       <c r="A23" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -990,29 +1028,29 @@
       <c r="G23" s="11"/>
       <c r="H23" s="11"/>
       <c r="I23" s="3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="J23" s="3"/>
     </row>
     <row r="24" spans="1:10" ht="18.45" customHeight="1">
       <c r="A24" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H24" s="3"/>
       <c r="I24" s="3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="J24" s="3"/>
     </row>
@@ -1030,7 +1068,7 @@
     </row>
     <row r="26" spans="1:10" ht="22.35" customHeight="1">
       <c r="A26" s="12" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B26" s="12"/>
       <c r="C26" s="12"/>
@@ -1044,7 +1082,7 @@
     </row>
     <row r="27" spans="1:10" ht="22.35" customHeight="1">
       <c r="A27" s="12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12"/>
@@ -1071,24 +1109,24 @@
     <mergeCell ref="A16:A20"/>
     <mergeCell ref="A21:A22"/>
     <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C9:D9"/>
     <mergeCell ref="F18:J18"/>
     <mergeCell ref="C19:D19"/>
     <mergeCell ref="F19:J19"/>
     <mergeCell ref="C20:D20"/>
     <mergeCell ref="F20:J20"/>
-    <mergeCell ref="C15:D15"/>
     <mergeCell ref="F15:J15"/>
     <mergeCell ref="C16:D16"/>
     <mergeCell ref="F16:J16"/>
     <mergeCell ref="C17:D17"/>
     <mergeCell ref="F17:J17"/>
-    <mergeCell ref="C12:D12"/>
     <mergeCell ref="F12:J12"/>
     <mergeCell ref="C13:D13"/>
     <mergeCell ref="F13:J13"/>
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="F14:J14"/>
-    <mergeCell ref="C9:D9"/>
     <mergeCell ref="F9:J9"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="F10:J10"/>
@@ -1097,8 +1135,8 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:J1"/>
     <mergeCell ref="B5:F5"/>
+    <mergeCell ref="F8:J8"/>
     <mergeCell ref="C8:D8"/>
-    <mergeCell ref="F8:J8"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>